<commit_message>
Add MMHC Voordaan to clubs list
</commit_message>
<xml_diff>
--- a/hockeyclubs_nederland.xlsx
+++ b/hockeyclubs_nederland.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E280"/>
+  <dimension ref="A1:E281"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5159,9 +5159,26 @@
         <v>Joure</v>
       </c>
     </row>
+    <row r="281">
+      <c r="A281">
+        <v>280</v>
+      </c>
+      <c r="B281" t="str">
+        <v>Voordaan (M.M.H.C.)</v>
+      </c>
+      <c r="C281" t="str">
+        <v>Lindenlaan 66A</v>
+      </c>
+      <c r="D281" t="str">
+        <v>3737 RD</v>
+      </c>
+      <c r="E281" t="str">
+        <v>Groenekan</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E280"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E281"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>